<commit_message>
Atelier des vilains, custom-dio rejouable + cartes Dio interactives
Snapshot du travail local en cours avant fusion avec origin/main :
- Atelier des vilains (editeur) : onglets cartes/plateau/quantite, import
  Excel, export assets, layouts cartes (recto/dos), stores custom.
- Dio Brando recree comme vilain custom (custom-dio) : remappage vers ids
  natifs + reinjection des effets/champs de jeu (customDio.ts).
- Cartes Dio a choix rendues INTERACTIVES (pending + modale ; bot auto) :
  Vampirisme, Justice, CREAM, MUDA, Quete vers le paradis, Lumiere du Soleil.
  Effet DIO_RECOVER_ALLY_FROM_DISCARD supprime. Tests customDio.test.ts.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/decks/Villainous_Template-Alexis_1_1.xlsx
+++ b/assets/decks/Villainous_Template-Alexis_1_1.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\villainous\Villainous Card Localizer V28\Villainous Card Generator_Data\-TextFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC-Alexis\villainous\assets\decks\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{431EBE83-6E97-4DEE-B813-AD35CD32B8F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -5474,7 +5474,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="24" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" ht="36.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>20</v>
       </c>
@@ -5505,7 +5505,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="24" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" ht="36.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>16</v>
       </c>
@@ -5689,7 +5689,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="24" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" ht="36.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>22</v>
       </c>
@@ -6340,7 +6340,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:26" s="10" customFormat="1" ht="54.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:26" s="10" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="6">
         <v>2</v>
       </c>
@@ -24002,7 +24002,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="72.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" ht="54.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27" s="6">
         <v>1</v>
       </c>
@@ -24913,7 +24913,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="108.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" ht="90.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="6">
         <v>2</v>
       </c>
@@ -29785,7 +29785,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="23" spans="1:13" s="10" customFormat="1" ht="90.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" s="10" customFormat="1" ht="108.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>16</v>
       </c>
@@ -29967,7 +29967,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:13" s="10" customFormat="1" ht="24" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" s="10" customFormat="1" ht="36.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>16</v>
       </c>
@@ -30083,7 +30083,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="33" spans="1:13" s="10" customFormat="1" ht="24" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" s="10" customFormat="1" ht="36.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>16</v>
       </c>
@@ -34632,7 +34632,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="24" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27" s="6">
         <v>2</v>
       </c>
@@ -37545,7 +37545,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="23" spans="1:13" s="10" customFormat="1" ht="54.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" s="10" customFormat="1" ht="72.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="6">
         <v>1</v>
       </c>
@@ -37576,7 +37576,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:13" s="10" customFormat="1" ht="54.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" s="10" customFormat="1" ht="72.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6">
         <v>1</v>
       </c>
@@ -37607,7 +37607,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:13" s="10" customFormat="1" ht="24" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" s="10" customFormat="1" ht="36.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="6">
         <v>3</v>
       </c>
@@ -43263,7 +43263,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:13" s="5" customFormat="1" ht="72.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" s="5" customFormat="1" ht="54.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="6">
         <v>2</v>
       </c>
@@ -43449,7 +43449,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:13" s="5" customFormat="1" ht="24" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" s="5" customFormat="1" ht="36.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="6">
         <v>2</v>
       </c>
@@ -43600,7 +43600,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="1:13" s="5" customFormat="1" ht="24" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" s="5" customFormat="1" ht="36.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="6">
         <v>2</v>
       </c>
@@ -43629,7 +43629,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:13" s="5" customFormat="1" ht="24" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" s="5" customFormat="1" ht="36.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="6">
         <v>2</v>
       </c>
@@ -43658,7 +43658,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="1:13" s="5" customFormat="1" ht="24" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" s="5" customFormat="1" ht="36.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="6">
         <v>2</v>
       </c>
@@ -46407,7 +46407,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:13" s="10" customFormat="1" ht="54.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" s="10" customFormat="1" ht="72.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6">
         <v>2</v>
       </c>
@@ -46562,7 +46562,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="1:13" s="10" customFormat="1" ht="54.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" s="10" customFormat="1" ht="72.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="6">
         <v>1</v>
       </c>
@@ -46655,7 +46655,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="28" spans="1:13" s="10" customFormat="1" ht="24" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" s="10" customFormat="1" ht="36.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A28" s="6">
         <v>2</v>
       </c>
@@ -46684,7 +46684,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:13" s="10" customFormat="1" ht="24" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" s="10" customFormat="1" ht="36.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A29" s="6">
         <v>2</v>
       </c>
@@ -46713,7 +46713,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="1:13" s="10" customFormat="1" ht="24" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" s="10" customFormat="1" ht="36.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A30" s="6">
         <v>2</v>
       </c>
@@ -46742,7 +46742,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:13" s="10" customFormat="1" ht="24" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" s="10" customFormat="1" ht="36.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A31" s="6">
         <v>2</v>
       </c>
@@ -49239,7 +49239,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:13" s="10" customFormat="1" ht="90.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" s="10" customFormat="1" ht="72.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="6">
         <v>2</v>
       </c>
@@ -49642,7 +49642,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="1:13" s="10" customFormat="1" ht="24" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" s="10" customFormat="1" ht="36.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="6">
         <v>2</v>
       </c>

</xml_diff>